<commit_message>
James Walker's rulings of 23 September: SDWS 26 served share is the seasonal average; scale mapping confirmed; piped usage survey action; days operational per system with a 1 km service unit
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/action_owners.xlsx
+++ b/build/action_owners.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -748,7 +748,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the 7-point gap between the MadAvance dashboard and our register.</t>
+          <t>Reconcile the gap between the MadAvance dashboard and our register.</t>
         </is>
       </c>
     </row>
@@ -1679,283 +1679,280 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>act-point-use-round-one</t>
+          <t>act-piped-usage-survey</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MadAvance / Cathy</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Point-of-use round one.</t>
+          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>act-population-rerun</t>
+          <t>act-point-use-round-one</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>MadAvance / Cathy</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Re-run the population model whenever the portfolio grows.</t>
+          <t>Point-of-use round one.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>act-printed-year-meaning</t>
+          <t>act-population-rerun</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="n">
-        <v>46312</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
+          <t>Re-run the population model whenever the portfolio grows.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>act-produce-s4-19-cl</t>
+          <t>act-printed-year-meaning</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Adriaan, submitted by James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Produce the installation database.</t>
+          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>act-put-current-methodology-vpa</t>
+          <t>act-produce-s4-19-cl</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Adriaan, submitted by James Walker</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
-        <v>46295</v>
+        <v>46326</v>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
+          <t>Produce the installation database.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>act-put-usage-question-live</t>
+          <t>act-put-current-methodology-vpa</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Adriaan / MadAvance</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>46295</v>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
+          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>act-re-run-improved-cookstove</t>
+          <t>act-put-usage-question-live</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Adriaan / MadAvance</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Re-run the improved-cookstove usage question every year.</t>
+          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>act-reconcile-cookstove-water-programmes</t>
+          <t>act-re-run-improved-cookstove</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Angelo, tracked by Jan</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the cookstove and water programmes for double counting.</t>
+          <t>Re-run the improved-cookstove usage question every year.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>act-recreate-gardien-calendar-controlled</t>
+          <t>act-reconcile-cookstove-water-programmes</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="n">
-        <v>46326</v>
+          <t>James Walker on method, Adriaan on data</t>
+        </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Recreate the gardien calendar as a controlled document.</t>
+          <t>Reconcile the cookstove and water programmes for double counting.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>act-reduced-performance</t>
+          <t>act-recreate-gardien-calendar-controlled</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
+          <t>Recreate the gardien calendar as a controlled document.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>act-refresh-extract</t>
+          <t>act-reduced-performance</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Refresh the mWater extract before each edition.</t>
+          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>act-rehab-recording</t>
+          <t>act-refresh-extract</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="n">
-        <v>46298</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds 7 and 7.</t>
+          <t>Refresh the mWater extract before each edition.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>act-reissue-calendars-new-blank</t>
+          <t>act-rehab-recording</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Jan with Angelo</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C80" s="3" t="n">
-        <v>46387</v>
+        <v>46298</v>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
+          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds 7 and 7.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>act-repair-double-entry</t>
+          <t>act-reissue-calendars-new-blank</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Lanja Rakotomalala</t>
-        </is>
+          <t>Jan with Angelo</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="n">
+        <v>46387</v>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Decide what to do with one repair recorded twice across the form migration.</t>
+          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>act-repair-time</t>
+          <t>act-repair-double-entry</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="n">
-        <v>46387</v>
+          <t>Lanja Rakotomalala</t>
+        </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
+          <t>Decide what to do with one repair recorded twice across the form migration.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>act-repeat-breakdown</t>
+          <t>act-repair-time</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1963,56 +1960,56 @@
           <t>Jan de Graaf</t>
         </is>
       </c>
+      <c r="C83" s="3" t="n">
+        <v>46387</v>
+      </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
+          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-sdws-27-sdws</t>
+          <t>act-repeat-breakdown</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="n">
-        <v>46310</v>
+          <t>Jan de Graaf</t>
+        </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
+          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-water-point-type</t>
+          <t>act-resolve-sdws-27-sdws</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C85" s="3" t="n">
-        <v>46326</v>
+        <v>46310</v>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Resolve the water point type contradiction on 987623517.</t>
+          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>act-restore-preventive-maintenance-visit</t>
+          <t>act-resolve-water-point-type</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2021,78 +2018,78 @@
         </is>
       </c>
       <c r="C86" s="3" t="n">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
+          <t>Resolve the water point type contradiction on 987623517.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>act-retrain-field-teams-how</t>
+          <t>act-restore-preventive-maintenance-visit</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Angelo</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C87" s="3" t="n">
-        <v>46326</v>
+        <v>46356</v>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Retrain field teams on how to photograph the calendar.</t>
+          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>act-route-plans</t>
+          <t>act-retrain-field-teams-how</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Angelo</t>
         </is>
       </c>
       <c r="C88" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Build catch-up route plans for Fort-Dauphin and Marolinta.</t>
+          <t>Retrain field teams on how to photograph the calendar.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>act-run-sdws-26-premises</t>
+          <t>act-route-plans</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
+          <t>Build catch-up route plans for Fort-Dauphin and Marolinta.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>act-run-stroke-test-sdws</t>
+          <t>act-run-sdws-26-premises</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2101,69 +2098,72 @@
         </is>
       </c>
       <c r="C90" s="3" t="n">
-        <v>46371</v>
+        <v>46326</v>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
+          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-annual-round</t>
+          <t>act-run-stroke-test-sdws</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara, MadAvance water team</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="n">
+        <v>46371</v>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
+          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-approve-2025</t>
+          <t>act-sdws26-annual-round</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MadAvance</t>
+          <t>Angelo Nahavitatsara, MadAvance water team</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Approve the November 2025 usage responses in mWater.</t>
+          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-instrument-review</t>
+          <t>act-sdws26-approve-2025</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>MadAvance</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
+          <t>Approve the November 2025 usage responses in mWater.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>act-sdws27-basis</t>
+          <t>act-sdws26-instrument-review</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2171,198 +2171,195 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C94" s="3" t="n">
-        <v>46298</v>
-      </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Settle the SDWS 27 basis with Gold Standard.</t>
+          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>act-sdws3-operating-status</t>
+          <t>act-sdws27-basis</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C95" s="3" t="n">
-        <v>46312</v>
+        <v>46298</v>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
+          <t>Settle the SDWS 27 basis with Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-definition</t>
+          <t>act-sdws3-operating-status</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C96" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Put the sensor definition to Gold Standard.</t>
+          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-sample</t>
+          <t>act-sensor-definition</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
+          <t>Put the sensor definition to Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>act-settle-baseline-boiling-device</t>
+          <t>act-sensor-sample</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C98" s="3" t="n">
-        <v>46356</v>
+        <v>46298</v>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
+          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>act-standardised-stroke-test-basis</t>
+          <t>act-settle-baseline-boiling-device</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>James Walker on method, Adriaan on data</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="n">
+        <v>46356</v>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Standardised stroke test — the basis is settled.</t>
+          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>act-transcription-round</t>
+          <t>act-standardised-stroke-test-basis</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MadAvance — transcriber to be named</t>
-        </is>
-      </c>
-      <c r="C100" s="3" t="n">
-        <v>46305</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Run the transcription validation round.</t>
+          <t>Standardised stroke test — the basis is settled.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>act-type3-cap</t>
+          <t>act-transcription-round</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>MadAvance — transcriber to be named</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
+          <t>Run the transcription validation round.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>act-undatable</t>
+          <t>act-type3-cap</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C102" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Quantify the water points behind the 395 undatable sheets, and merge with the reissue list.</t>
+          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>act-update-parameters-workbook-cite</t>
+          <t>act-undatable</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Update the parameters workbook to cite the applied basis.</t>
+          <t>Quantify the water points behind the 395 undatable sheets, and merge with the reissue list.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>act-update-sops-portfolio-figures</t>
+          <t>act-update-parameters-workbook-cite</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C104" s="3" t="n">
@@ -2370,31 +2367,34 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Update the SOP’s portfolio figures.</t>
+          <t>Update the parameters workbook to cite the applied basis.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>act-v2-adherence</t>
+          <t>act-update-sops-portfolio-figures</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Methodology version adherence — standing item.</t>
+          <t>Update the SOP’s portfolio figures.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>act-v2-confidence-intervals</t>
+          <t>act-v2-adherence</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2402,19 +2402,16 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C106" s="3" t="n">
-        <v>46312</v>
-      </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
+          <t>Methodology version adherence — standing item.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>act-v2-embodied</t>
+          <t>act-v2-confidence-intervals</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2423,18 +2420,18 @@
         </is>
       </c>
       <c r="C107" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Start recording commissioning year and technology category as a monitoring output.</t>
+          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>act-v2-nonclaiming</t>
+          <t>act-v2-embodied</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2443,18 +2440,18 @@
         </is>
       </c>
       <c r="C108" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
+          <t>Start recording commissioning year and technology category as a monitoring output.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>act-v2-sample-size</t>
+          <t>act-v2-nonclaiming</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2463,18 +2460,18 @@
         </is>
       </c>
       <c r="C109" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Re-scope every sample against the v2.0 minimum of 50.</t>
+          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stove-stacking</t>
+          <t>act-v2-sample-size</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2483,18 +2480,18 @@
         </is>
       </c>
       <c r="C110" s="3" t="n">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Add a stove-stacking question to the annual monitoring survey.</t>
+          <t>Re-scope every sample against the v2.0 minimum of 50.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stroke-test</t>
+          <t>act-v2-stove-stacking</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2503,66 +2500,86 @@
         </is>
       </c>
       <c r="C111" s="3" t="n">
-        <v>46305</v>
+        <v>46326</v>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+          <t>Add a stove-stacking question to the annual monitoring survey.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>act-visit-collapse</t>
+          <t>act-v2-stroke-test</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C112" s="3" t="n">
-        <v>46295</v>
+        <v>46305</v>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>act-visit-three-marolinta-points</t>
+          <t>act-visit-collapse</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
-        <v>46387</v>
+        <v>46295</v>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
+          <t>act-visit-three-marolinta-points</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
           <t>act-wq-retest</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
-      <c r="D114" s="4" t="inlineStr">
+      <c r="D115" s="4" t="inlineStr">
         <is>
           <t>Confirm the one failed E. coli test was retested.</t>
         </is>
@@ -2570,10 +2587,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
+    <dataValidation sqref="B2:B115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
       <formula1>"Adriaan Mol,James Walker,Jan de Graaf,Angelo Nahavitatsara,Lanja Randriamanantena,MadAvance,Angelo Nahavitatsara / MadAvance,Lanja Randriamanantena / MadAvance,MadAvance field teams,Jan / Endur'O team,Coddy,Cathy,Earthood,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C114" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
       <formula1>DATE(2024,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2687,7 +2704,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seeded 2026-09-23 from 113 actions by tools/make_owner_workbook.py</t>
+          <t>Seeded 2026-09-25 from 114 actions by tools/make_owner_workbook.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Piped systems join the managed portfolio only after works and post-rehabilitation tests; the Amboasary gara results are pre-project baseline and count toward no managed figure
Adriaan Mol, 25 September 2026. data/piped_systems_status.json gives every
Endur'O water system a status; the four Moramanga systems (Amboasary gara,
Ambohibola, Amboanjo, Andilanatoby) are identified from the Moramanga baseline
survey and identification forms and are in process. rebuild_piped_wq.py keys
the rule on result date against works completion, so a system joins on its own
and its baseline results never count; tools/test_piped_wq.py proves it. The
build fails on an Endur'O system with no status. The 30 km proxy is withdrawn.
Two actions: the misfiled Sainte Luce results (Lanja), and post-rehabilitation
tests with the sampled tap recorded (Jan with Endur'O). The mWater tooling pin
now names its private remote, SaniTap-water/mwater-mcp.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/action_owners.xlsx
+++ b/build/action_owners.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -631,7 +631,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Close out the 6.5% residual against the January population run.</t>
+          <t>Close out the unexplained residual against the January population run.</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Confirm the Maroantsetra fNRB value at 34%.</t>
+          <t>Confirm the Maroantsetra fNRB value at %.</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Decide how to treat the 67 points with no usable calendar image: exclude, or estimate.</t>
+          <t>Decide how to treat the points with no usable calendar image: exclude, or estimate.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Record where the 146,000 Endur'O people figure comes from.</t>
+          <t>Record where the Endur'O people figure comes from.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Settle the India Mark premises figure — 500 or 300.</t>
+          <t>Settle the India Mark premises figure — or .</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Record the 3 rehabilitations that have no record at all.</t>
+          <t>Record the rehabilitations that have no record at all.</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Record the 4 new boreholes that have no record at all.</t>
+          <t>Record the new boreholes that have no record at all.</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Correct the village spelling on 19 works-form records.</t>
+          <t>Correct the village spelling on the works-form records that spell it Marolita.</t>
         </is>
       </c>
     </row>
@@ -1498,148 +1498,145 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Submit the 4 draft new-construction records on the Moramanga deployment.</t>
+          <t>Submit the draft new-construction records on the Moramanga deployment.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>act-move-stroke-test-sop</t>
+          <t>act-moramanga-post-rehab-wq</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf with Endur’O</t>
+        </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Move the stroke-test SOP into the SOPs folder and get it signed off.</t>
+          <t>Post-rehabilitation water-quality tests on the four Moramanga piped systems; record the sampled tap on every result.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>act-move-weekly-mwater-backup</t>
+          <t>act-move-stroke-test-sop</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Adriaan</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Move the weekly mWater backup off the laptop.</t>
+          <t>Move the stroke-test SOP into the SOPs folder and get it signed off.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-approval-policy</t>
+          <t>act-move-weekly-mwater-backup</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan</t>
+        </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
+          <t>Move the weekly mWater backup off the laptop.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-mg-locale</t>
+          <t>act-mwater-approval-policy</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
+          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>46298</v>
+        <v>46326</v>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
+          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-year-required</t>
+          <t>act-mwater-mg-locale</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
-        <v>46418</v>
+        <v>46298</v>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
+          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>act-no-works-record</t>
+          <t>act-mwater-year-required</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>46418</v>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
+          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>act-per-diem</t>
+          <t>act-no-works-record</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="n">
-        <v>46326</v>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
+          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>act-photo-conditional-on-presence</t>
+          <t>act-per-diem</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1648,18 +1645,18 @@
         </is>
       </c>
       <c r="C66" s="3" t="n">
-        <v>46286</v>
+        <v>46326</v>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
+          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>act-photo-misfiled</t>
+          <t>act-photo-conditional-on-presence</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1668,234 +1665,240 @@
         </is>
       </c>
       <c r="C67" s="3" t="n">
-        <v>46326</v>
+        <v>46286</v>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Move the 206 misfiled photographs to the question they belong on.</t>
+          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>act-piped-usage-survey</t>
+          <t>act-photo-misfiled</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
+          <t>Move the misfiled photographs to the question they belong on.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>act-point-use-round-one</t>
+          <t>act-piped-usage-survey</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MadAvance / Cathy</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Point-of-use round one.</t>
+          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>act-population-rerun</t>
+          <t>act-piped-wq-misfiled-742895333</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Lanja Randriamanantena / MadAvance</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Re-run the population model whenever the portfolio grows.</t>
+          <t xml:space="preserve">Two water-quality results for hand pump 742895333 (Sainte Luce) were filed on the piped results form 0ac68d82; re-enter </t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>act-printed-year-meaning</t>
+          <t>act-point-use-round-one</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="n">
-        <v>46312</v>
+          <t>MadAvance / Cathy</t>
+        </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
+          <t>Point-of-use round one.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>act-produce-s4-19-cl</t>
+          <t>act-population-rerun</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Adriaan, submitted by James Walker</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Produce the installation database.</t>
+          <t>Re-run the population model whenever the portfolio grows.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>act-put-current-methodology-vpa</t>
+          <t>act-printed-year-meaning</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
-        <v>46295</v>
+        <v>46312</v>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
+          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>act-put-usage-question-live</t>
+          <t>act-produce-s4-19-cl</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Adriaan / MadAvance</t>
-        </is>
+          <t>Adriaan, submitted by James Walker</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
+          <t>Produce the installation database.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>act-re-run-improved-cookstove</t>
+          <t>act-put-current-methodology-vpa</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>46295</v>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Re-run the improved-cookstove usage question every year.</t>
+          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>act-reconcile-cookstove-water-programmes</t>
+          <t>act-put-usage-question-live</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Adriaan / MadAvance</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the cookstove and water programmes for double counting.</t>
+          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>act-recreate-gardien-calendar-controlled</t>
+          <t>act-re-run-improved-cookstove</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="n">
-        <v>46326</v>
+          <t>Angelo, tracked by Jan</t>
+        </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Recreate the gardien calendar as a controlled document.</t>
+          <t>Re-run the improved-cookstove usage question every year.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>act-reduced-performance</t>
+          <t>act-reconcile-cookstove-water-programmes</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>James Walker on method, Adriaan on data</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
+          <t>Reconcile the cookstove and water programmes for double counting.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>act-refresh-extract</t>
+          <t>act-recreate-gardien-calendar-controlled</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Refresh the mWater extract before each edition.</t>
+          <t>Recreate the gardien calendar as a controlled document.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>act-rehab-recording</t>
+          <t>act-reduced-performance</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1903,61 +1906,58 @@
           <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
-      <c r="C80" s="3" t="n">
-        <v>46298</v>
-      </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds 7 and 7.</t>
+          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>act-reissue-calendars-new-blank</t>
+          <t>act-refresh-extract</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Jan with Angelo</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="n">
-        <v>46387</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
+          <t>Refresh the mWater extract before each edition.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>act-repair-double-entry</t>
+          <t>act-rehab-recording</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Lanja Rakotomalala</t>
-        </is>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Decide what to do with one repair recorded twice across the form migration.</t>
+          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds and .</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>act-repair-time</t>
+          <t>act-reissue-calendars-new-blank</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan with Angelo</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
@@ -1965,96 +1965,93 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
+          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>act-repeat-breakdown</t>
+          <t>act-repair-double-entry</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Lanja Rakotomalala</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
+          <t>Decide what to do with one repair recorded twice across the form migration.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-sdws-27-sdws</t>
+          <t>act-repair-time</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C85" s="3" t="n">
-        <v>46310</v>
+        <v>46387</v>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
+          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-water-point-type</t>
+          <t>act-repeat-breakdown</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C86" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf</t>
+        </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Resolve the water point type contradiction on 987623517.</t>
+          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>act-restore-preventive-maintenance-visit</t>
+          <t>act-resolve-sdws-27-sdws</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C87" s="3" t="n">
-        <v>46356</v>
+        <v>46310</v>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
+          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>act-retrain-field-teams-how</t>
+          <t>act-resolve-water-point-type</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Angelo</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C88" s="3" t="n">
@@ -2062,39 +2059,39 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Retrain field teams on how to photograph the calendar.</t>
+          <t>Resolve the water point type contradiction on 987623517.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>act-route-plans</t>
+          <t>act-restore-preventive-maintenance-visit</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
-        <v>46312</v>
+        <v>46356</v>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Build catch-up route plans for Fort-Dauphin and Marolinta.</t>
+          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>act-run-sdws-26-premises</t>
+          <t>act-retrain-field-teams-how</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Angelo</t>
         </is>
       </c>
       <c r="C90" s="3" t="n">
@@ -2102,125 +2099,125 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
+          <t>Retrain field teams on how to photograph the calendar.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>act-run-stroke-test-sdws</t>
+          <t>act-route-plans</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
-        <v>46371</v>
+        <v>46312</v>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
+          <t>Build a catch-up route plan for Marolinta, and keep Fort-Dauphin’s current.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-annual-round</t>
+          <t>act-run-sdws-26-premises</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara, MadAvance water team</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
+          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-approve-2025</t>
+          <t>act-run-stroke-test-sdws</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="n">
+        <v>46371</v>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Approve the November 2025 usage responses in mWater.</t>
+          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-instrument-review</t>
+          <t>act-sdws26-annual-round</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara, MadAvance water team</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
+          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>act-sdws27-basis</t>
+          <t>act-sdws26-approve-2025</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C95" s="3" t="n">
-        <v>46298</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Settle the SDWS 27 basis with Gold Standard.</t>
+          <t>Approve the November 2025 usage responses in mWater.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>act-sdws3-operating-status</t>
+          <t>act-sdws26-instrument-review</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
+          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-definition</t>
+          <t>act-sdws27-basis</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2229,18 +2226,18 @@
         </is>
       </c>
       <c r="C97" s="3" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Put the sensor definition to Gold Standard.</t>
+          <t>Settle the SDWS 27 basis with Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-sample</t>
+          <t>act-sdws3-operating-status</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2249,112 +2246,115 @@
         </is>
       </c>
       <c r="C98" s="3" t="n">
-        <v>46298</v>
+        <v>46312</v>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
+          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>act-settle-baseline-boiling-device</t>
+          <t>act-sensor-definition</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
-        <v>46356</v>
+        <v>46305</v>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
+          <t>Put the sensor definition to Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>act-standardised-stroke-test-basis</t>
+          <t>act-sensor-sample</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Standardised stroke test — the basis is settled.</t>
+          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>act-transcription-round</t>
+          <t>act-settle-baseline-boiling-device</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MadAvance — transcriber to be named</t>
+          <t>James Walker on method, Adriaan on data</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
-        <v>46305</v>
+        <v>46356</v>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Run the transcription validation round.</t>
+          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>act-type3-cap</t>
+          <t>act-standardised-stroke-test-basis</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>MadAvance</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
+          <t>Standardised stroke test — the basis is settled.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>act-undatable</t>
+          <t>act-transcription-round</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>MadAvance — transcriber to be named</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Quantify the water points behind the 395 undatable sheets, and merge with the reissue list.</t>
+          <t>Run the transcription validation round.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>act-update-parameters-workbook-cite</t>
+          <t>act-type3-cap</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2362,39 +2362,36 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C104" s="3" t="n">
-        <v>46326</v>
-      </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Update the parameters workbook to cite the applied basis.</t>
+          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>act-update-sops-portfolio-figures</t>
+          <t>act-undatable</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C105" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Update the SOP’s portfolio figures.</t>
+          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>act-v2-adherence</t>
+          <t>act-update-parameters-workbook-cite</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2402,36 +2399,39 @@
           <t>James Walker</t>
         </is>
       </c>
+      <c r="C106" s="3" t="n">
+        <v>46326</v>
+      </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Methodology version adherence — standing item.</t>
+          <t>Update the parameters workbook to cite the applied basis.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>act-v2-confidence-intervals</t>
+          <t>act-update-sops-portfolio-figures</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
+          <t>Update the SOP’s portfolio figures.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>act-v2-embodied</t>
+          <t>act-v2-adherence</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2439,19 +2439,16 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C108" s="3" t="n">
-        <v>46326</v>
-      </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Start recording commissioning year and technology category as a monitoring output.</t>
+          <t>Methodology version adherence — standing item.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>act-v2-nonclaiming</t>
+          <t>act-v2-confidence-intervals</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2464,14 +2461,14 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
+          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>act-v2-sample-size</t>
+          <t>act-v2-embodied</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2480,18 +2477,18 @@
         </is>
       </c>
       <c r="C110" s="3" t="n">
-        <v>46305</v>
+        <v>46326</v>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Re-scope every sample against the v2.0 minimum of 50.</t>
+          <t>Start recording commissioning year and technology category as a monitoring output.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stove-stacking</t>
+          <t>act-v2-nonclaiming</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2500,18 +2497,18 @@
         </is>
       </c>
       <c r="C111" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Add a stove-stacking question to the annual monitoring survey.</t>
+          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stroke-test</t>
+          <t>act-v2-sample-size</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2524,62 +2521,102 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+          <t>Re-scope every sample against the v2.0 minimum of .</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>act-visit-collapse</t>
+          <t>act-v2-stove-stacking</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
-        <v>46295</v>
+        <v>46326</v>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+          <t>Add a stove-stacking question to the annual monitoring survey.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>act-visit-three-marolinta-points</t>
+          <t>act-v2-stroke-test</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C114" s="3" t="n">
-        <v>46387</v>
+        <v>46305</v>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
+          <t>act-visit-collapse</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Jan de Graaf</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>act-visit-three-marolinta-points</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
           <t>act-wq-retest</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
-      <c r="D115" s="4" t="inlineStr">
+      <c r="D117" s="4" t="inlineStr">
         <is>
           <t>Confirm the one failed E. coli test was retested.</t>
         </is>
@@ -2587,10 +2624,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
+    <dataValidation sqref="B2:B117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
       <formula1>"Adriaan Mol,James Walker,Jan de Graaf,Angelo Nahavitatsara,Lanja Randriamanantena,MadAvance,Angelo Nahavitatsara / MadAvance,Lanja Randriamanantena / MadAvance,MadAvance field teams,Jan / Endur'O team,Coddy,Cathy,Earthood,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
       <formula1>DATE(2024,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2704,7 +2741,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seeded 2026-09-25 from 114 actions by tools/make_owner_workbook.py</t>
+          <t>Seeded 2026-09-25 from 116 actions by tools/make_owner_workbook.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
James Walker's replies of 18, 21 and 23 Sep: Maroantsetra fNRB applied at 36% beside the registered 34%, nine actions closed with their sources, seven annotated, four added, SOP versions beside the originals, and the VPA-DD copied into the Methodology of record
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/action_owners.xlsx
+++ b/build/action_owners.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -812,72 +812,69 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>act-down-no-repair</t>
+          <t>act-design-change-q1-2027</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker, data by Adriaan</t>
+        </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Close the call-centre down reports that have no repair record.</t>
+          <t>Design change with the Q1 2027 verification: apply v2.0 to 2025, and correct the VPA-DD.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>act-duplicate-codes-sweep</t>
+          <t>act-down-no-repair</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>46286</v>
+        <v>46312</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Clear the six duplicated question codes on the other three forms.</t>
+          <t>Close the call-centre down reports that have no repair record.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>act-emergency-event-form</t>
+          <t>act-duplicate-codes-sweep</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>46326</v>
+        <v>46286</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Settle where SDWS 3 emergency-event evidence is actually recorded — the form the SOP names does not exist.</t>
+          <t>Clear the six duplicated question codes on the other three forms.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-feed</t>
+          <t>act-emergency-event-form</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -885,19 +882,19 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: a dispensing-events feed from Curtech — device id, timestamp, litres, card and credits for every dis</t>
+          <t>Settle where SDWS 3 emergency-event evidence is actually recorded — the form the SOP names does not exist.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-move-register-fully</t>
+          <t>act-enduro-feed</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jan, with Coddy</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -905,59 +902,59 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding into mWater: move the register fully into mWater, in seven steps.</t>
+          <t>Endur’O onboarding: a dispensing-events feed from Curtech — device id, timestamp, litres, card and credits for every dis</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-1-enumerators</t>
+          <t>act-enduro-move-register-fully</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coddy</t>
+          <t>Jan, with Coddy</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>46298</v>
+        <v>46326</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: populate the enumerator team so the two registration forms open in the field app.</t>
+          <t>Endur’O onboarding into mWater: move the register fully into mWater, in seven steps.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-2-register-sites</t>
+          <t>act-enduro-onboard-1-enumerators</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Coddy with Jan</t>
+          <t>Coddy</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>46326</v>
+        <v>46298</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: register every managed Endur’O site with the System and Distribution Point forms.</t>
+          <t>Endur’O onboarding: populate the enumerator team so the two registration forms open in the field app.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-3-bind-taps</t>
+          <t>act-enduro-onboard-2-register-sites</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Coddy</t>
+          <t>Coddy with Jan</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -965,19 +962,19 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: bind every smart tap to its water point by the paired-timestamp test dispense.</t>
+          <t>Endur’O onboarding: register every managed Endur’O site with the System and Distribution Point forms.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-5-calibration</t>
+          <t>act-enduro-onboard-3-bind-taps</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ralf van Veenendaal (Curtech)</t>
+          <t>Coddy</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -985,71 +982,74 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endur’O onboarding: a calibration certificate for every installed meter, traceable to its device id (Gold Standard SDWS </t>
+          <t>Endur’O onboarding: bind every smart tap to its water point by the paired-timestamp test dispense.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-6-kiosk-wq</t>
+          <t>act-enduro-onboard-5-calibration</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jan de Graaf with Cathy Andriambololonirina (Mandie)</t>
+          <t>Ralf van Veenendaal (Curtech)</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>46311</v>
+        <v>46326</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: a water-quality test at the dispensing point of the managed kiosk, bound to the water point, not the</t>
+          <t xml:space="preserve">Endur’O onboarding: a calibration certificate for every installed meter, traceable to its device id (Gold Standard SDWS </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-onboard-7-piped-sdws27</t>
+          <t>act-enduro-onboard-6-kiosk-wq</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Coddy with Jan</t>
+          <t>Jan de Graaf with Cathy Andriambololonirina (Mandie)</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>46326</v>
+        <v>46311</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Endur’O onboarding: piped maintenance, repair and days-not-operational records in mWater — the SDWS 27 evidence.</t>
+          <t>Endur’O onboarding: a water-quality test at the dispensing point of the managed kiosk, bound to the water point, not the</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-people-source</t>
+          <t>act-enduro-onboard-7-piped-sdws27</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Coddy with Jan</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Record where the Endur'O people figure comes from.</t>
+          <t>Endur’O onboarding: piped maintenance, repair and days-not-operational records in mWater — the SDWS 27 evidence.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>act-enduro-refresh</t>
+          <t>act-enduro-people-source</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1059,34 +1059,31 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Re-confirm the hand-entered Endur'O figures.</t>
+          <t>Record where the Endur'O people figure comes from.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>act-establish-renewal-dates-current</t>
+          <t>act-enduro-refresh</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Establish renewal dates and current status for the four baseline parameters.</t>
+          <t>Re-confirm the hand-entered Endur'O figures.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>act-establish-renewal-dates-four</t>
+          <t>act-establish-renewal-dates-current</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1094,166 +1091,166 @@
           <t>James Walker</t>
         </is>
       </c>
+      <c r="C34" s="3" t="n">
+        <v>46326</v>
+      </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Establish renewal dates for the four baseline parameters.</t>
+          <t>Establish renewal dates and current status for the four baseline parameters.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>act-figure-residue</t>
+          <t>act-establish-renewal-dates-four</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Resolve the remaining unsourced figures.</t>
+          <t>Establish renewal dates for the four baseline parameters.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>act-find-source-annual-independent</t>
+          <t>act-figure-residue</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Adriaan</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Find a source for the annual independent cross-check of people per premises.</t>
+          <t>Resolve the remaining unsourced figures.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>act-fleet-growth</t>
+          <t>act-find-source-annual-independent</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="n">
-        <v>46312</v>
+          <t>Adriaan</t>
+        </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>The carbon fleet has not grown in nine months. Establish what the pipeline actually is.</t>
+          <t>Find a source for the annual independent cross-check of people per premises.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>act-form-consolidation</t>
+          <t>act-fleet-growth</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Jan de Graaf</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>46312</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Decide whether to consolidate the Marolinta borehole form into the works form.</t>
+          <t>The carbon fleet has not grown in nine months. Establish what the pipeline actually is.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>act-freeze-estate-map-when</t>
+          <t>act-form-consolidation</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Adriaan</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Freeze the estate map when an edition is archived.</t>
+          <t>Decide whether to consolidate the Marolinta borehole form into the works form.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>act-gaps-doc</t>
+          <t>act-freeze-estate-map-when</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>46298</v>
+          <t>Adriaan</t>
+        </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Correct the carbon-data-gaps source document: it says the cookstove overlap has not been calculated, and it has.</t>
+          <t>Freeze the estate map when an edition is archived.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>act-identify-count-institutional-premises</t>
+          <t>act-gaps-doc</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Jan de Graaf</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Identify and count institutional premises inside the service areas.</t>
+          <t>Correct the carbon-data-gaps source document: it says the cookstove overlap has not been calculated, and it has.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>act-indiamark-premises</t>
+          <t>act-identify-count-institutional-premises</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>46326</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Settle the India Mark premises figure — or .</t>
+          <t>Identify and count institutional premises inside the service areas.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>act-make-calendar-photograph-mandatory</t>
+          <t>act-indiamark-premises</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Lanja</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
@@ -1261,65 +1258,68 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Make the calendar photograph a mandatory field on both visit forms.</t>
+          <t>Settle the India Mark premises figure — or .</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>act-mar-admin-fields</t>
+          <t>act-make-calendar-photograph-mandatory</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Lanja</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Set the administrative fields and pump model on the Marolinta records in mWater.</t>
+          <t>Make the calendar photograph a mandatory field on both visit forms.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>act-mar-functional-status</t>
+          <t>act-mar-admin-fields</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Fill “Statut fonctionnel actuel” on the new-construction records.</t>
+          <t>Set the administrative fields and pump model on the Marolinta records in mWater.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>act-mar-missing-boreholes</t>
+          <t>act-mar-functional-status</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Enter the Marolinta new-borehole records that are missing.</t>
+          <t>Fill “Statut fonctionnel actuel” on the new-construction records.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>act-mar-missing-rehabs</t>
+          <t>act-mar-missing-boreholes</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1329,14 +1329,14 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Record the rehabilitations that have no record at all.</t>
+          <t>Enter the Marolinta new-borehole records that are missing.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>act-mar-new-construction-gap</t>
+          <t>act-mar-missing-rehabs</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1346,14 +1346,14 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Record the new boreholes that have no record at all.</t>
+          <t>Record the rehabilitations that have no record at all.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>act-mar-technical-values</t>
+          <t>act-mar-new-construction-gap</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1363,82 +1363,82 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Check the repeated technical values with the drilling supervisor.</t>
+          <t>Record the new boreholes that have no record at all.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>act-mar-water-quality</t>
+          <t>act-mar-technical-values</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Get a passed E. coli test at the point of collection on every Marolinta borehole.</t>
+          <t>Check the repeated technical values with the drilling supervisor.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>act-mar-which-form</t>
+          <t>act-mar-water-quality</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Get the field teams onto the current first-rehabilitation form.</t>
+          <t>Get a passed E. coli test at the point of collection on every Marolinta borehole.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>act-marolita-spelling</t>
+          <t>act-mar-which-form</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Correct the village spelling on the works-form records that spell it Marolita.</t>
+          <t>Get the field teams onto the current first-rehabilitation form.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>act-mor-1b-betanatanana-go-look</t>
+          <t>act-marolita-spelling</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jan / Endur’O team</t>
+          <t>Angelo Nahavitatsara</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>1b. Betanatanana — go and look at this well</t>
+          <t>Correct the village spelling on the works-form records that spell it Marolita.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>act-mor-bring-back-site-lists</t>
+          <t>act-mor-1b-betanatanana-go-look</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1448,14 +1448,14 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>10. Bring back site lists with coordinates for Andaingo and Fieferana / Manjakandriana</t>
+          <t>1b. Betanatanana — go and look at this well</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>act-mor-correct-two-sampling-records</t>
+          <t>act-mor-bring-back-site-lists</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1465,14 +1465,14 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>8. Correct two sampling records</t>
+          <t>10. Bring back site lists with coordinates for Andaingo and Fieferana / Manjakandriana</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>act-mor-count-draw-off-point</t>
+          <t>act-mor-correct-two-sampling-records</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1482,14 +1482,14 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>3. Count every draw-off point on the system</t>
+          <t>8. Correct two sampling records</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>act-mor-fill-three-new-fields</t>
+          <t>act-mor-count-draw-off-point</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1499,14 +1499,14 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>9. Fill the three new fields on the results form from the next round</t>
+          <t>3. Count every draw-off point on the system</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>act-mor-fix-type-sampled-point</t>
+          <t>act-mor-fill-three-new-fields</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1516,14 +1516,14 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>4. Fix the type of each sampled point, once</t>
+          <t>9. Fill the three new fields on the results form from the next round</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>act-mor-have-those-five-records</t>
+          <t>act-mor-fix-type-sampled-point</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1533,14 +1533,14 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>2. Have those five records shared with SaniTap</t>
+          <t>4. Fix the type of each sampled point, once</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>act-mor-households-people-served-per</t>
+          <t>act-mor-have-those-five-records</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1550,14 +1550,14 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>5. Households and people served per draw-off point</t>
+          <t>2. Have those five records shared with SaniTap</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>act-mor-re-take-gps-fix</t>
+          <t>act-mor-households-people-served-per</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1567,14 +1567,14 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1. Re-take the GPS fix at Amboasary Gara</t>
+          <t>5. Households and people served per draw-off point</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>act-mor-record-what-community-drank</t>
+          <t>act-mor-re-take-gps-fix</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1584,14 +1584,14 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>6. Record what each community drank before the system</t>
+          <t>1. Re-take the GPS fix at Amboasary Gara</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>act-mor-remove-reclassify-two-test</t>
+          <t>act-mor-record-what-community-drank</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1601,14 +1601,14 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>7. Remove or reclassify two test records in the hand-pump register</t>
+          <t>6. Record what each community drank before the system</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>act-mor-submit-drafts</t>
+          <t>act-mor-remove-reclassify-two-test</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1618,165 +1618,162 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Submit the draft new-construction records on the Moramanga deployment.</t>
+          <t>7. Remove or reclassify two test records in the hand-pump register</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>act-moramanga-post-rehab-wq</t>
+          <t>act-mor-submit-drafts</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Jan de Graaf with Endur’O</t>
+          <t>Jan / Endur’O team</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Post-rehabilitation water-quality tests on the four Moramanga piped systems; record the sampled tap on every result.</t>
+          <t>Submit the draft new-construction records on the Moramanga deployment.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>act-move-stroke-test-sop</t>
+          <t>act-moramanga-post-rehab-wq</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf with Endur’O</t>
+        </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Move the stroke-test SOP into the SOPs folder and get it signed off.</t>
+          <t>Post-rehabilitation water-quality tests on the four Moramanga piped systems; record the sampled tap on every result.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>act-move-weekly-mwater-backup</t>
+          <t>act-move-stroke-test-sop</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Adriaan</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Move the weekly mWater backup off the laptop.</t>
+          <t>Move the stroke-test SOP into the SOPs folder and get it signed off.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-approval-policy</t>
+          <t>act-move-weekly-mwater-backup</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan</t>
+        </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
+          <t>Move the weekly mWater backup off the laptop.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-mg-locale</t>
+          <t>act-mwater-approval-policy</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
+          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
-        <v>46298</v>
+        <v>46326</v>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
+          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-year-required</t>
+          <t>act-mwater-mg-locale</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
-        <v>46418</v>
+        <v>46298</v>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
+          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>act-no-works-record</t>
+          <t>act-mwater-year-required</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="n">
+        <v>46418</v>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
+          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>act-per-diem</t>
+          <t>act-no-works-record</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="n">
-        <v>46326</v>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
+          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>act-photo-conditional-on-presence</t>
+          <t>act-per-diem</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1785,18 +1782,18 @@
         </is>
       </c>
       <c r="C73" s="3" t="n">
-        <v>46286</v>
+        <v>46326</v>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
+          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>act-photo-misfiled</t>
+          <t>act-photo-conditional-on-presence</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1805,254 +1802,257 @@
         </is>
       </c>
       <c r="C74" s="3" t="n">
-        <v>46326</v>
+        <v>46286</v>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Move the misfiled photographs to the question they belong on.</t>
+          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>act-piped-usage-survey</t>
+          <t>act-photo-misfiled</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
+          <t>Move the misfiled photographs to the question they belong on.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>act-piped-wq-misfiled-742895333</t>
+          <t>act-piped-fnrb</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="n">
-        <v>46305</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two water-quality results for hand pump 742895333 (Sainte Luce) were filed on the piped results form 0ac68d82; re-enter </t>
+          <t>Settle the fNRB for the piped VPA before its VPA-DD is submitted.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>act-point-use-round-one</t>
+          <t>act-piped-usage-survey</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MadAvance / Cathy</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Point-of-use round one.</t>
+          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>act-population-rerun</t>
+          <t>act-piped-wq-misfiled-742895333</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Lanja Randriamanantena / MadAvance</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Re-run the population model whenever the portfolio grows.</t>
+          <t xml:space="preserve">Two water-quality results for hand pump 742895333 (Sainte Luce) were filed on the piped results form 0ac68d82; re-enter </t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>act-printed-year-meaning</t>
+          <t>act-point-use-round-one</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="n">
-        <v>46312</v>
+          <t>MadAvance / Cathy</t>
+        </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
+          <t>Point-of-use round one.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>act-produce-s4-19-cl</t>
+          <t>act-population-rerun</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Adriaan, submitted by James Walker</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Produce the installation database.</t>
+          <t>Re-run the population model whenever the portfolio grows.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>act-put-current-methodology-vpa</t>
+          <t>act-printed-year-meaning</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
-        <v>46295</v>
+        <v>46312</v>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
+          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>act-put-usage-question-live</t>
+          <t>act-produce-s4-19-cl</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Adriaan / MadAvance</t>
-        </is>
+          <t>Adriaan, submitted by James Walker</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
+          <t>Produce the installation database.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>act-re-run-improved-cookstove</t>
+          <t>act-put-current-methodology-vpa</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>46295</v>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Re-run the improved-cookstove usage question every year.</t>
+          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>act-reconcile-cookstove-water-programmes</t>
+          <t>act-put-usage-question-live</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Adriaan / MadAvance</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the cookstove and water programmes for double counting.</t>
+          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>act-recreate-gardien-calendar-controlled</t>
+          <t>act-re-run-improved-cookstove</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="n">
-        <v>46326</v>
+          <t>Angelo, tracked by Jan</t>
+        </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Recreate the gardien calendar as a controlled document.</t>
+          <t>Re-run the improved-cookstove usage question every year.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>act-reduced-performance</t>
+          <t>act-reconcile-cookstove-water-programmes</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>James Walker on method, Adriaan on data</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
+          <t>Reconcile the cookstove and water programmes for double counting.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>act-refresh-extract</t>
+          <t>act-recreate-gardien-calendar-controlled</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Refresh the mWater extract before each edition.</t>
+          <t>Recreate the gardien calendar as a controlled document.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>act-rehab-recording</t>
+          <t>act-reduced-performance</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2060,61 +2060,58 @@
           <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
-      <c r="C88" s="3" t="n">
-        <v>46298</v>
-      </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds and .</t>
+          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>act-reissue-calendars-new-blank</t>
+          <t>act-refresh-extract</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Jan with Angelo</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="n">
-        <v>46387</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
+          <t>Refresh the mWater extract before each edition.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>act-repair-double-entry</t>
+          <t>act-rehab-recording</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Lanja Rakotomalala</t>
-        </is>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Decide what to do with one repair recorded twice across the form migration.</t>
+          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds and .</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>act-repair-time</t>
+          <t>act-reissue-calendars-new-blank</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan with Angelo</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
@@ -2122,96 +2119,93 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
+          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>act-repeat-breakdown</t>
+          <t>act-repair-double-entry</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Lanja Randriamanantena</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
+          <t>Decide what to do with one repair recorded twice across the form migration.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-sdws-27-sdws</t>
+          <t>act-repair-time</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
-        <v>46310</v>
+        <v>46387</v>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
+          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-water-point-type</t>
+          <t>act-repeat-breakdown</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C94" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf</t>
+        </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Resolve the water point type contradiction on 987623517.</t>
+          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>act-restore-preventive-maintenance-visit</t>
+          <t>act-resolve-sdws-27-sdws</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C95" s="3" t="n">
-        <v>46356</v>
+        <v>46310</v>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
+          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>act-retrain-field-teams-how</t>
+          <t>act-resolve-water-point-type</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Angelo</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C96" s="3" t="n">
@@ -2219,39 +2213,39 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Retrain field teams on how to photograph the calendar.</t>
+          <t>Resolve the water point type contradiction on 987623517.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>act-route-plans</t>
+          <t>act-restore-preventive-maintenance-visit</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
-        <v>46312</v>
+        <v>46356</v>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Build a catch-up route plan for Marolinta, and keep Fort-Dauphin’s current.</t>
+          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>act-run-sdws-26-premises</t>
+          <t>act-retrain-field-teams-how</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Angelo</t>
         </is>
       </c>
       <c r="C98" s="3" t="n">
@@ -2259,125 +2253,125 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
+          <t>Retrain field teams on how to photograph the calendar.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>act-run-stroke-test-sdws</t>
+          <t>act-route-plans</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
-        <v>46371</v>
+        <v>46312</v>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
+          <t>Build a catch-up route plan for Marolinta, and keep Fort-Dauphin’s current.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-annual-round</t>
+          <t>act-run-sdws-26-premises</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara, MadAvance water team</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
+          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-approve-2025</t>
+          <t>act-run-stroke-test-sdws</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>46371</v>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Approve the November 2025 usage responses in mWater.</t>
+          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-instrument-review</t>
+          <t>act-sdws26-annual-round</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara, MadAvance water team</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
+          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>act-sdws27-basis</t>
+          <t>act-sdws26-approve-2025</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C103" s="3" t="n">
-        <v>46298</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Settle the SDWS 27 basis with Gold Standard.</t>
+          <t>Approve the November 2025 usage responses in mWater.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>act-sdws3-operating-status</t>
+          <t>act-sdws26-instrument-review</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C104" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
+          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-definition</t>
+          <t>act-sdws27-basis</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2386,18 +2380,18 @@
         </is>
       </c>
       <c r="C105" s="3" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Put the sensor definition to Gold Standard.</t>
+          <t>Settle the SDWS 27 basis with Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-sample</t>
+          <t>act-sdws3-operating-status</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2406,169 +2400,172 @@
         </is>
       </c>
       <c r="C106" s="3" t="n">
-        <v>46298</v>
+        <v>46312</v>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
+          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>act-settle-baseline-boiling-device</t>
+          <t>act-sensor-cost-benefit</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
-        <v>46356</v>
+        <v>46326</v>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
+          <t>Cost-benefit of a sensor on every pump against the sample of 100.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>act-standardised-stroke-test-basis</t>
+          <t>act-sensor-definition</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Standardised stroke test — the basis is settled.</t>
+          <t>Put the sensor definition to Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>act-transcription-round</t>
+          <t>act-sensor-sample</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MadAvance — transcriber to be named</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C109" s="3" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Run the transcription validation round.</t>
+          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>act-type3-cap</t>
+          <t>act-settle-baseline-boiling-device</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>James Walker on method, Adriaan on data</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>46356</v>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
+          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>act-undatable</t>
+          <t>act-standardised-stroke-test-basis</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C111" s="3" t="n">
-        <v>46312</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
+          <t>Standardised stroke test — the basis is settled.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>act-update-parameters-workbook-cite</t>
+          <t>act-transcription-round</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>MadAvance — transcriber to be named</t>
         </is>
       </c>
       <c r="C112" s="3" t="n">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Update the parameters workbook to cite the applied basis.</t>
+          <t>Run the transcription validation round.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>act-update-sops-portfolio-figures</t>
+          <t>act-type3-cap</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="n">
-        <v>46326</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Update the SOP’s portfolio figures.</t>
+          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>act-v2-adherence</t>
+          <t>act-undatable</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>46312</v>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Methodology version adherence — standing item.</t>
+          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>act-v2-confidence-intervals</t>
+          <t>act-update-parameters-workbook-cite</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2577,23 +2574,23 @@
         </is>
       </c>
       <c r="C115" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
+          <t>Update the parameters workbook to cite the applied basis.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>act-v2-embodied</t>
+          <t>act-update-sops-portfolio-figures</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C116" s="3" t="n">
@@ -2601,14 +2598,14 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Start recording commissioning year and technology category as a monitoring output.</t>
+          <t>Update the SOP’s portfolio figures.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>act-v2-nonclaiming</t>
+          <t>act-v2-adherence</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2616,19 +2613,16 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C117" s="3" t="n">
-        <v>46312</v>
-      </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
+          <t>Methodology version adherence — standing item.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>act-v2-sample-size</t>
+          <t>act-v2-confidence-intervals</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2637,18 +2631,18 @@
         </is>
       </c>
       <c r="C118" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Re-scope every sample against the v2.0 minimum of .</t>
+          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stove-stacking</t>
+          <t>act-v2-embodied</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2661,14 +2655,14 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Add a stove-stacking question to the annual monitoring survey.</t>
+          <t>Start recording commissioning year and technology category as a monitoring output.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stroke-test</t>
+          <t>act-v2-nonclaiming</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2677,66 +2671,143 @@
         </is>
       </c>
       <c r="C120" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>act-visit-collapse</t>
+          <t>act-v2-sample-size</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C121" s="3" t="n">
-        <v>46295</v>
+        <v>46305</v>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+          <t>Re-scope every sample against the v2.0 minimum of .</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>act-visit-three-marolinta-points</t>
+          <t>act-v2-stove-stacking</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C122" s="3" t="n">
-        <v>46387</v>
+        <v>46326</v>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+          <t>Add a stove-stacking question to the annual monitoring survey.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
+          <t>act-v2-stroke-test</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>act-verification-fnrb-correction</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Include the Maroantsetra fNRB correction in the Q1 2027 verification submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>act-visit-collapse</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Jan de Graaf</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>act-visit-three-marolinta-points</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
           <t>act-wq-retest</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
-      <c r="D123" s="4" t="inlineStr">
+      <c r="D127" s="4" t="inlineStr">
         <is>
           <t>Confirm the one failed E. coli test was retested.</t>
         </is>
@@ -2744,10 +2815,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
+    <dataValidation sqref="B2:B127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
       <formula1>"Adriaan Mol,James Walker,Jan de Graaf,Angelo Nahavitatsara,Lanja Randriamanantena,MadAvance,Angelo Nahavitatsara / MadAvance,Lanja Randriamanantena / MadAvance,MadAvance field teams,Jan / Endur'O team,Coddy,Cathy,Earthood,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
       <formula1>DATE(2024,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2861,7 +2932,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seeded 2026-09-26 from 122 actions by tools/make_owner_workbook.py</t>
+          <t>Seeded 2026-09-26 from 126 actions by tools/make_owner_workbook.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sign-off actions for the new SOP versions: calendar v1.7 added for Angelo, stroke-test v2.1 merged into act-move-stroke-test-sop and closing on a logged decision; the Curtech StrokeMeter briefing noted as drafted 26 Sep, awaiting send
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/action_owners.xlsx
+++ b/build/action_owners.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Move the stroke-test SOP into the SOPs folder and get it signed off.</t>
+          <t>Approve stroke-test SOP v2.1 in French and English, move the French version into the SOPs folder, and retire v2.0.</t>
         </is>
       </c>
     </row>
@@ -2491,106 +2491,106 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>act-standardised-stroke-test-basis</t>
+          <t>act-sop-calendar-v17-signoff</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Standardised stroke test — the basis is settled.</t>
+          <t>Approve calendar SOP v1.7, brief every field team on it in French, then retire v1.6.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>act-transcription-round</t>
+          <t>act-standardised-stroke-test-basis</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MadAvance — transcriber to be named</t>
-        </is>
-      </c>
-      <c r="C112" s="3" t="n">
-        <v>46305</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Run the transcription validation round.</t>
+          <t>Standardised stroke test — the basis is settled.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>act-type3-cap</t>
+          <t>act-transcription-round</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>MadAvance — transcriber to be named</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
+          <t>Run the transcription validation round.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>act-undatable</t>
+          <t>act-type3-cap</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C114" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
+          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>act-update-parameters-workbook-cite</t>
+          <t>act-undatable</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C115" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Update the parameters workbook to cite the applied basis.</t>
+          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>act-update-sops-portfolio-figures</t>
+          <t>act-update-parameters-workbook-cite</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C116" s="3" t="n">
@@ -2598,31 +2598,34 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Update the SOP’s portfolio figures.</t>
+          <t>Update the parameters workbook to cite the applied basis.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>act-v2-adherence</t>
+          <t>act-update-sops-portfolio-figures</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Methodology version adherence — standing item.</t>
+          <t>Update the SOP’s portfolio figures.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>act-v2-confidence-intervals</t>
+          <t>act-v2-adherence</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2630,19 +2633,16 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C118" s="3" t="n">
-        <v>46312</v>
-      </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
+          <t>Methodology version adherence — standing item.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>act-v2-embodied</t>
+          <t>act-v2-confidence-intervals</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2651,18 +2651,18 @@
         </is>
       </c>
       <c r="C119" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Start recording commissioning year and technology category as a monitoring output.</t>
+          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>act-v2-nonclaiming</t>
+          <t>act-v2-embodied</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2671,18 +2671,18 @@
         </is>
       </c>
       <c r="C120" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
+          <t>Start recording commissioning year and technology category as a monitoring output.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>act-v2-sample-size</t>
+          <t>act-v2-nonclaiming</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -2691,18 +2691,18 @@
         </is>
       </c>
       <c r="C121" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Re-scope every sample against the v2.0 minimum of .</t>
+          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stove-stacking</t>
+          <t>act-v2-sample-size</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -2711,18 +2711,18 @@
         </is>
       </c>
       <c r="C122" s="3" t="n">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Add a stove-stacking question to the annual monitoring survey.</t>
+          <t>Re-scope every sample against the v2.0 minimum of .</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stroke-test</t>
+          <t>act-v2-stove-stacking</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2731,18 +2731,18 @@
         </is>
       </c>
       <c r="C123" s="3" t="n">
-        <v>46305</v>
+        <v>46326</v>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+          <t>Add a stove-stacking question to the annual monitoring survey.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>act-verification-fnrb-correction</t>
+          <t>act-v2-stroke-test</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2750,64 +2750,84 @@
           <t>James Walker</t>
         </is>
       </c>
+      <c r="C124" s="3" t="n">
+        <v>46305</v>
+      </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>Include the Maroantsetra fNRB correction in the Q1 2027 verification submission.</t>
+          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>act-visit-collapse</t>
+          <t>act-verification-fnrb-correction</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C125" s="3" t="n">
-        <v>46295</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+          <t>Include the Maroantsetra fNRB correction in the Q1 2027 verification submission.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>act-visit-three-marolinta-points</t>
+          <t>act-visit-collapse</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C126" s="3" t="n">
-        <v>46387</v>
+        <v>46295</v>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
+          <t>act-visit-three-marolinta-points</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
           <t>act-wq-retest</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
-      <c r="D127" s="4" t="inlineStr">
+      <c r="D128" s="4" t="inlineStr">
         <is>
           <t>Confirm the one failed E. coli test was retested.</t>
         </is>
@@ -2815,10 +2835,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
+    <dataValidation sqref="B2:B128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
       <formula1>"Adriaan Mol,James Walker,Jan de Graaf,Angelo Nahavitatsara,Lanja Randriamanantena,MadAvance,Angelo Nahavitatsara / MadAvance,Lanja Randriamanantena / MadAvance,MadAvance field teams,Jan / Endur'O team,Coddy,Cathy,Earthood,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
       <formula1>DATE(2024,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2932,7 +2952,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seeded 2026-09-26 from 126 actions by tools/make_owner_workbook.py</t>
+          <t>Seeded 2026-09-26 from 127 actions by tools/make_owner_workbook.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
James Walker's reply of 21 Sep 2026 ("Re: Water program dashboard & actions"): the v2.0 stroke-test parameter is SDWS 28, not SDWS 27, and Gold Standard is expected to withdraw the quarterly Option 3 validation. act-resolve-sdws-27-sdws closed on the logged decision; act-gs-validation-withdrawal-watch and act-mwater-backup-restore-check added; progress noted on act-v2-confidence-intervals and act-enduro-onboard-5-calibration; stroke-test SOP v2.2 (FR and EN) beside v2.1; week 39 edition 9 archived first; extracts re-pulled 28 Sep; ACTN.overdue given its derivation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/action_owners.xlsx
+++ b/build/action_owners.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D128"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1228,49 +1228,49 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>act-identify-count-institutional-premises</t>
+          <t>act-gs-validation-withdrawal-watch</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>46387</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Identify and count institutional premises inside the service areas.</t>
+          <t>Watch for Gold Standard’s correction of the v2.0 quarterly Option 3 validation.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>act-indiamark-premises</t>
+          <t>act-identify-count-institutional-premises</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>46326</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Settle the India Mark premises figure — or .</t>
+          <t>Identify and count institutional premises inside the service areas.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>act-make-calendar-photograph-mandatory</t>
+          <t>act-indiamark-premises</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Lanja</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -1278,65 +1278,68 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Make the calendar photograph a mandatory field on both visit forms.</t>
+          <t>Settle the India Mark premises figure — or .</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>act-mar-admin-fields</t>
+          <t>act-make-calendar-photograph-mandatory</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Lanja</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Set the administrative fields and pump model on the Marolinta records in mWater.</t>
+          <t>Make the calendar photograph a mandatory field on both visit forms.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>act-mar-functional-status</t>
+          <t>act-mar-admin-fields</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Fill “Statut fonctionnel actuel” on the new-construction records.</t>
+          <t>Set the administrative fields and pump model on the Marolinta records in mWater.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>act-mar-missing-boreholes</t>
+          <t>act-mar-functional-status</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Enter the Marolinta new-borehole records that are missing.</t>
+          <t>Fill “Statut fonctionnel actuel” on the new-construction records.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>act-mar-missing-rehabs</t>
+          <t>act-mar-missing-boreholes</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1346,14 +1349,14 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Record the rehabilitations that have no record at all.</t>
+          <t>Enter the Marolinta new-borehole records that are missing.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>act-mar-new-construction-gap</t>
+          <t>act-mar-missing-rehabs</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1363,14 +1366,14 @@
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Record the new boreholes that have no record at all.</t>
+          <t>Record the rehabilitations that have no record at all.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>act-mar-technical-values</t>
+          <t>act-mar-new-construction-gap</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1380,82 +1383,82 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Check the repeated technical values with the drilling supervisor.</t>
+          <t>Record the new boreholes that have no record at all.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>act-mar-water-quality</t>
+          <t>act-mar-technical-values</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Get a passed E. coli test at the point of collection on every Marolinta borehole.</t>
+          <t>Check the repeated technical values with the drilling supervisor.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>act-mar-which-form</t>
+          <t>act-mar-water-quality</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Get the field teams onto the current first-rehabilitation form.</t>
+          <t>Get a passed E. coli test at the point of collection on every Marolinta borehole.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>act-marolita-spelling</t>
+          <t>act-mar-which-form</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Correct the village spelling on the works-form records that spell it Marolita.</t>
+          <t>Get the field teams onto the current first-rehabilitation form.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>act-mor-1b-betanatanana-go-look</t>
+          <t>act-marolita-spelling</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Jan / Endur’O team</t>
+          <t>Angelo Nahavitatsara</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>1b. Betanatanana — go and look at this well</t>
+          <t>Correct the village spelling on the works-form records that spell it Marolita.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>act-mor-bring-back-site-lists</t>
+          <t>act-mor-1b-betanatanana-go-look</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1465,14 +1468,14 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>10. Bring back site lists with coordinates for Andaingo and Fieferana / Manjakandriana</t>
+          <t>1b. Betanatanana — go and look at this well</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>act-mor-correct-two-sampling-records</t>
+          <t>act-mor-bring-back-site-lists</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1482,14 +1485,14 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>8. Correct two sampling records</t>
+          <t>10. Bring back site lists with coordinates for Andaingo and Fieferana / Manjakandriana</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>act-mor-count-draw-off-point</t>
+          <t>act-mor-correct-two-sampling-records</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1499,14 +1502,14 @@
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>3. Count every draw-off point on the system</t>
+          <t>8. Correct two sampling records</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>act-mor-fill-three-new-fields</t>
+          <t>act-mor-count-draw-off-point</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1516,14 +1519,14 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>9. Fill the three new fields on the results form from the next round</t>
+          <t>3. Count every draw-off point on the system</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>act-mor-fix-type-sampled-point</t>
+          <t>act-mor-fill-three-new-fields</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1533,14 +1536,14 @@
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>4. Fix the type of each sampled point, once</t>
+          <t>9. Fill the three new fields on the results form from the next round</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>act-mor-have-those-five-records</t>
+          <t>act-mor-fix-type-sampled-point</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1550,14 +1553,14 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2. Have those five records shared with SaniTap</t>
+          <t>4. Fix the type of each sampled point, once</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>act-mor-households-people-served-per</t>
+          <t>act-mor-have-those-five-records</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1567,14 +1570,14 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>5. Households and people served per draw-off point</t>
+          <t>2. Have those five records shared with SaniTap</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>act-mor-re-take-gps-fix</t>
+          <t>act-mor-households-people-served-per</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1584,14 +1587,14 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>1. Re-take the GPS fix at Amboasary Gara</t>
+          <t>5. Households and people served per draw-off point</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>act-mor-record-what-community-drank</t>
+          <t>act-mor-re-take-gps-fix</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1601,14 +1604,14 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>6. Record what each community drank before the system</t>
+          <t>1. Re-take the GPS fix at Amboasary Gara</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>act-mor-remove-reclassify-two-test</t>
+          <t>act-mor-record-what-community-drank</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1618,14 +1621,14 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>7. Remove or reclassify two test records in the hand-pump register</t>
+          <t>6. Record what each community drank before the system</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>act-mor-submit-drafts</t>
+          <t>act-mor-remove-reclassify-two-test</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1635,108 +1638,105 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Submit the draft new-construction records on the Moramanga deployment.</t>
+          <t>7. Remove or reclassify two test records in the hand-pump register</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>act-moramanga-post-rehab-wq</t>
+          <t>act-mor-submit-drafts</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jan de Graaf with Endur’O</t>
+          <t>Jan / Endur’O team</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Post-rehabilitation water-quality tests on the four Moramanga piped systems; record the sampled tap on every result.</t>
+          <t>Submit the draft new-construction records on the Moramanga deployment.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>act-move-stroke-test-sop</t>
+          <t>act-moramanga-post-rehab-wq</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf with Endur’O</t>
+        </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Approve stroke-test SOP v2.1 in French and English, move the French version into the SOPs folder, and retire v2.0.</t>
+          <t>Post-rehabilitation water-quality tests on the four Moramanga piped systems; record the sampled tap on every result.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>act-move-weekly-mwater-backup</t>
+          <t>act-move-stroke-test-sop</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Adriaan</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Move the weekly mWater backup off the laptop.</t>
+          <t>Approve stroke-test SOP v2.1 in French and English, move the French version into the SOPs folder, and retire v2.0.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-approval-policy</t>
+          <t>act-move-weekly-mwater-backup</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan</t>
+        </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
+          <t>Move the weekly mWater backup off the laptop.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-mg-locale</t>
+          <t>act-mwater-approval-policy</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
+          <t>Angelo Nahavitatsara / MadAvance with Jan de Graaf</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
-        <v>46298</v>
+        <v>46326</v>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
+          <t>Define what approving an mWater record means, then apply it only where it buys something.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>act-mwater-year-required</t>
+          <t>act-mwater-backup-restore-check</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1745,35 +1745,38 @@
         </is>
       </c>
       <c r="C71" s="3" t="n">
-        <v>46418</v>
+        <v>46297</v>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
+          <t>Check what the mWater backup restore brought back, and that nothing edited after it was lost.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>act-no-works-record</t>
+          <t>act-mwater-mg-locale</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
+          <t>Lanja Randriamanantena / MadAvance</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
+          <t>Add the Malagasy locale to the Entretien préventif form, so Malagasy labels stop having to lead the French string.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>act-per-diem</t>
+          <t>act-mwater-year-required</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1782,38 +1785,35 @@
         </is>
       </c>
       <c r="C73" s="3" t="n">
-        <v>46326</v>
+        <v>46418</v>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
+          <t>Make mWater question 2.15.7 required, once v1.4 stock and the SOP are in the field in both districts.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>act-photo-conditional-on-presence</t>
+          <t>act-no-works-record</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="n">
-        <v>46286</v>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
+          <t>Enter a works record, or remove from the register, for every point that has neither.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>act-photo-misfiled</t>
+          <t>act-per-diem</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1826,267 +1826,273 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Move the misfiled photographs to the question they belong on.</t>
+          <t>Redesign the per-diem system so it pays for pumps completed, not days in the field.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>act-piped-fnrb</t>
+          <t>act-photo-conditional-on-presence</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>46286</v>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Settle the fNRB for the piped VPA before its VPA-DD is submitted.</t>
+          <t>Make the calendar photograph conditional on a calendar being present on the repair-after-breakdown form, as it now is on</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>act-piped-usage-survey</t>
+          <t>act-photo-misfiled</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
+          <t>Adriaan Mol</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
+          <t>Move the misfiled photographs to the question they belong on.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>act-piped-wq-misfiled-742895333</t>
+          <t>act-piped-fnrb</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena / MadAvance</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="n">
-        <v>46305</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two water-quality results for hand pump 742895333 (Sainte Luce) were filed on the piped results form 0ac68d82; re-enter </t>
+          <t>Settle the fNRB for the piped VPA before its VPA-DD is submitted.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>act-point-use-round-one</t>
+          <t>act-piped-usage-survey</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MadAvance / Cathy</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Point-of-use round one.</t>
+          <t>Annual usage survey for the piped systems — separate from the hand-pump survey; JMP core questions, household size, usag</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>act-population-rerun</t>
+          <t>act-piped-wq-misfiled-742895333</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Lanja Randriamanantena / MadAvance</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="n">
+        <v>46305</v>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Re-run the population model whenever the portfolio grows.</t>
+          <t xml:space="preserve">Two water-quality results for hand pump 742895333 (Sainte Luce) were filed on the piped results form 0ac68d82; re-enter </t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>act-printed-year-meaning</t>
+          <t>act-point-use-round-one</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="n">
-        <v>46312</v>
+          <t>MadAvance / Cathy</t>
+        </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
+          <t>Point-of-use round one.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>act-produce-s4-19-cl</t>
+          <t>act-population-rerun</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Adriaan, submitted by James Walker</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="n">
-        <v>46326</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Produce the installation database.</t>
+          <t>Re-run the population model whenever the portfolio grows.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>act-put-current-methodology-vpa</t>
+          <t>act-printed-year-meaning</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
-        <v>46295</v>
+        <v>46312</v>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
+          <t>Establish what the year printed on a gardien calendar is meant to denote, and whether sheets are issued with a forward y</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>act-put-usage-question-live</t>
+          <t>act-produce-s4-19-cl</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Adriaan / MadAvance</t>
-        </is>
+          <t>Adriaan, submitted by James Walker</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
+          <t>Produce the installation database.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>act-re-run-improved-cookstove</t>
+          <t>act-put-current-methodology-vpa</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
-        </is>
+          <t>James Walker</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>46295</v>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Re-run the improved-cookstove usage question every year.</t>
+          <t>Put the current methodology and our VPA-DD into the Central Data Hub.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>act-reconcile-cookstove-water-programmes</t>
+          <t>act-put-usage-question-live</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>Adriaan / MadAvance</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the cookstove and water programmes for double counting.</t>
+          <t>Put the usage question on a live mWater form and run usage survey round one.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>act-recreate-gardien-calendar-controlled</t>
+          <t>act-re-run-improved-cookstove</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C87" s="3" t="n">
-        <v>46326</v>
+          <t>Angelo, tracked by Jan</t>
+        </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Recreate the gardien calendar as a controlled document.</t>
+          <t>Re-run the improved-cookstove usage question every year.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>act-reduced-performance</t>
+          <t>act-reconcile-cookstove-water-programmes</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>James Walker on method, Adriaan on data</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
+          <t>Reconcile the cookstove and water programmes for double counting.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>act-refresh-extract</t>
+          <t>act-recreate-gardien-calendar-controlled</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>Refresh the mWater extract before each edition.</t>
+          <t>Recreate the gardien calendar as a controlled document.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>act-rehab-recording</t>
+          <t>act-reduced-performance</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2094,61 +2100,58 @@
           <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
-      <c r="C90" s="3" t="n">
-        <v>46298</v>
-      </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds and .</t>
+          <t>Check the pumps reported with reduced performance that are still counted as working.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>act-reissue-calendars-new-blank</t>
+          <t>act-refresh-extract</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Jan with Angelo</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="n">
-        <v>46387</v>
+          <t>Adriaan Mol</t>
+        </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
+          <t>Refresh the mWater extract before each edition.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>act-repair-double-entry</t>
+          <t>act-rehab-recording</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Lanja Randriamanantena</t>
-        </is>
+          <t>Angelo Nahavitatsara / MadAvance</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>46298</v>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>Decide what to do with one repair recorded twice across the form migration.</t>
+          <t>Reconcile the Marolinta count: the minutes say 10 and 10, the form holds and .</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>act-repair-time</t>
+          <t>act-reissue-calendars-new-blank</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan with Angelo</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
@@ -2156,96 +2159,93 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
+          <t>Reissue calendars on the new blank template, on visits already scheduled.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>act-repeat-breakdown</t>
+          <t>act-repair-double-entry</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Lanja Randriamanantena</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
+          <t>Decide what to do with one repair recorded twice across the form migration.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-sdws-27-sdws</t>
+          <t>act-repair-time</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C95" s="3" t="n">
-        <v>46310</v>
+        <v>46387</v>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
+          <t>Call-centre response and report-back time — an operational performance target, explicitly not a carbon figure.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>act-resolve-water-point-type</t>
+          <t>act-repeat-breakdown</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Jan</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="n">
-        <v>46326</v>
+          <t>Jan de Graaf</t>
+        </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>Resolve the water point type contradiction on 987623517.</t>
+          <t>Decide whether the two repeat-breakdown pumps need a second water point rather than a fifteenth repair.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>act-restore-preventive-maintenance-visit</t>
+          <t>act-resolve-sdws-27-sdws</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
-        <v>46356</v>
+        <v>46310</v>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
+          <t>Resolve the SDWS 27 / SDWS 28 numbering, and the calibration requirement.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>act-retrain-field-teams-how</t>
+          <t>act-resolve-water-point-type</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Angelo</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C98" s="3" t="n">
@@ -2253,39 +2253,39 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Retrain field teams on how to photograph the calendar.</t>
+          <t>Resolve the water point type contradiction on 987623517.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>act-route-plans</t>
+          <t>act-restore-preventive-maintenance-visit</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
-        <v>46312</v>
+        <v>46356</v>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>Build a catch-up route plan for Marolinta, and keep Fort-Dauphin’s current.</t>
+          <t>Restore the preventive-maintenance visit rate (SDWS 27).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>act-run-sdws-26-premises</t>
+          <t>act-retrain-field-teams-how</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Angelo</t>
         </is>
       </c>
       <c r="C100" s="3" t="n">
@@ -2293,165 +2293,165 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
+          <t>Retrain field teams on how to photograph the calendar.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>act-run-stroke-test-sdws</t>
+          <t>act-route-plans</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
+          <t>Jan de Graaf</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
-        <v>46371</v>
+        <v>46312</v>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
+          <t>Build a catch-up route plan for Marolinta, and keep Fort-Dauphin’s current.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-annual-round</t>
+          <t>act-run-sdws-26-premises</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara, MadAvance water team</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
+          <t>Run the SDWS 26 premises-served survey, and report the precision actually achieved.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-approve-2025</t>
+          <t>act-run-stroke-test-sdws</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>46371</v>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>Approve the November 2025 usage responses in mWater.</t>
+          <t>Run the stroke test on the SDWS 23 sample, to the SOP.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>act-sdws26-instrument-review</t>
+          <t>act-sdws26-annual-round</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Angelo Nahavitatsara, MadAvance water team</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
+          <t>Run the SDWS 26 usage round every year, and fix the cluster shortfall.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>act-sdws27-basis</t>
+          <t>act-sdws26-approve-2025</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>James Walker</t>
-        </is>
-      </c>
-      <c r="C105" s="3" t="n">
-        <v>46298</v>
+          <t>MadAvance</t>
+        </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>Settle the SDWS 27 basis with Gold Standard.</t>
+          <t>Approve the November 2025 usage responses in mWater.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>act-sdws3-operating-status</t>
+          <t>act-sdws26-instrument-review</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
-        </is>
-      </c>
-      <c r="C106" s="3" t="n">
-        <v>46312</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
+          <t>Review and sign off the SDWS 26 usage instrument before the field round.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-cost-benefit</t>
+          <t>act-sdws27-basis</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Adriaan Mol</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
-        <v>46326</v>
+        <v>46298</v>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Cost-benefit of a sensor on every pump against the sample of 100.</t>
+          <t>Settle the SDWS 27 basis with Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-definition</t>
+          <t>act-sdws3-operating-status</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C108" s="3" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Put the sensor definition to Gold Standard.</t>
+          <t>Add an operating-status question to the SDWS 3 water-quality forms.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>act-sensor-sample</t>
+          <t>act-sensor-cost-benefit</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2460,80 +2460,83 @@
         </is>
       </c>
       <c r="C109" s="3" t="n">
-        <v>46298</v>
+        <v>46326</v>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
+          <t>Cost-benefit of a sensor on every pump against the sample of 100.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>act-settle-baseline-boiling-device</t>
+          <t>act-sensor-definition</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>James Walker on method, Adriaan on data</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C110" s="3" t="n">
-        <v>46356</v>
+        <v>46305</v>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
+          <t>Put the sensor definition to Gold Standard.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>act-sop-calendar-v17-signoff</t>
+          <t>act-sensor-sample</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>Adriaan Mol</t>
         </is>
       </c>
       <c r="C111" s="3" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Approve calendar SOP v1.7, brief every field team on it in French, then retire v1.6.</t>
+          <t>Brief Ralf van Veenendaal at Curtech on the fleet-wide unit count and the calibration sample — they are two different nu</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>act-standardised-stroke-test-basis</t>
+          <t>act-settle-baseline-boiling-device</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MadAvance</t>
-        </is>
+          <t>James Walker on method, Adriaan on data</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>46356</v>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Standardised stroke test — the basis is settled.</t>
+          <t>Settle the baseline boiling device for stove-holding households in Anosy.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>act-transcription-round</t>
+          <t>act-sop-calendar-v17-signoff</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MadAvance — transcriber to be named</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
@@ -2541,51 +2544,51 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>Run the transcription validation round.</t>
+          <t>Approve calendar SOP v1.7, brief every field team on it in French, then retire v1.6.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>act-type3-cap</t>
+          <t>act-standardised-stroke-test-basis</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>MadAvance</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
+          <t>Standardised stroke test — the basis is settled.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>act-undatable</t>
+          <t>act-transcription-round</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Angelo Nahavitatsara / MadAvance</t>
+          <t>MadAvance — transcriber to be named</t>
         </is>
       </c>
       <c r="C115" s="3" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
+          <t>Run the transcription validation round.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>act-update-parameters-workbook-cite</t>
+          <t>act-type3-cap</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -2593,39 +2596,36 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C116" s="3" t="n">
-        <v>46326</v>
-      </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Update the parameters workbook to cite the applied basis.</t>
+          <t>Decide the route before the point count reaches the small-scale Type 3 annual cap.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>act-update-sops-portfolio-figures</t>
+          <t>act-undatable</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Angelo Nahavitatsara / MadAvance</t>
         </is>
       </c>
       <c r="C117" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>Update the SOP’s portfolio figures.</t>
+          <t>Quantify the water points behind the undatable sheets, and merge with the reissue list.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>act-v2-adherence</t>
+          <t>act-update-parameters-workbook-cite</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2633,36 +2633,39 @@
           <t>James Walker</t>
         </is>
       </c>
+      <c r="C118" s="3" t="n">
+        <v>46326</v>
+      </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Methodology version adherence — standing item.</t>
+          <t>Update the parameters workbook to cite the applied basis.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>act-v2-confidence-intervals</t>
+          <t>act-update-sops-portfolio-figures</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>James Walker</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C119" s="3" t="n">
-        <v>46312</v>
+        <v>46326</v>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
+          <t>Update the SOP’s portfolio figures.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>act-v2-embodied</t>
+          <t>act-v2-adherence</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2670,19 +2673,16 @@
           <t>James Walker</t>
         </is>
       </c>
-      <c r="C120" s="3" t="n">
-        <v>46326</v>
-      </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Start recording commissioning year and technology category as a monitoring output.</t>
+          <t>Methodology version adherence — standing item.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>act-v2-nonclaiming</t>
+          <t>act-v2-confidence-intervals</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -2695,14 +2695,14 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
+          <t>Retain confidence intervals, not just point estimates, on every sampled parameter from now on.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>act-v2-sample-size</t>
+          <t>act-v2-embodied</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -2711,18 +2711,18 @@
         </is>
       </c>
       <c r="C122" s="3" t="n">
-        <v>46305</v>
+        <v>46326</v>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Re-scope every sample against the v2.0 minimum of .</t>
+          <t>Start recording commissioning year and technology category as a monitoring output.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stove-stacking</t>
+          <t>act-v2-nonclaiming</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2731,18 +2731,18 @@
         </is>
       </c>
       <c r="C123" s="3" t="n">
-        <v>46326</v>
+        <v>46312</v>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>Add a stove-stacking question to the annual monitoring survey.</t>
+          <t>Close the individual-level consent gap — the community-level notice is already in place.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>act-v2-stroke-test</t>
+          <t>act-v2-sample-size</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2755,14 +2755,14 @@
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
+          <t>Re-scope every sample against the v2.0 minimum of .</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>act-verification-fnrb-correction</t>
+          <t>act-v2-stove-stacking</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2770,64 +2770,104 @@
           <t>James Walker</t>
         </is>
       </c>
+      <c r="C125" s="3" t="n">
+        <v>46326</v>
+      </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>Include the Maroantsetra fNRB correction in the Q1 2027 verification submission.</t>
+          <t>Add a stove-stacking question to the annual monitoring survey.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>act-visit-collapse</t>
+          <t>act-v2-stroke-test</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Jan de Graaf</t>
+          <t>James Walker</t>
         </is>
       </c>
       <c r="C126" s="3" t="n">
-        <v>46295</v>
+        <v>46305</v>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+          <t>Reconcile the stroke-test SOP with v2.0, which recognises it and adds a condition.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>act-visit-three-marolinta-points</t>
+          <t>act-verification-fnrb-correction</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Angelo, tracked by Jan</t>
-        </is>
-      </c>
-      <c r="C127" s="3" t="n">
-        <v>46387</v>
+          <t>James Walker</t>
+        </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+          <t>Include the Maroantsetra fNRB correction in the Q1 2027 verification submission.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
+          <t>act-visit-collapse</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Jan de Graaf</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>Maintenance visit frequency has collapsed, and calendar coverage depends on it directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>act-visit-three-marolinta-points</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Angelo, tracked by Jan</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="n">
+        <v>46387</v>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>Visit the three Marolinta points that have no photograph of any kind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
           <t>act-wq-retest</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t>Lanja Randriamanantena / MadAvance</t>
         </is>
       </c>
-      <c r="D128" s="4" t="inlineStr">
+      <c r="D130" s="4" t="inlineStr">
         <is>
           <t>Confirm the one failed E. coli test was retested.</t>
         </is>
@@ -2835,10 +2875,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
+    <dataValidation sqref="B2:B130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick an owner from the list, or add them to tools/make_owner_workbook.py" type="list">
       <formula1>"Adriaan Mol,James Walker,Jan de Graaf,Angelo Nahavitatsara,Lanja Randriamanantena,MadAvance,Angelo Nahavitatsara / MadAvance,Lanja Randriamanantena / MadAvance,MadAvance field teams,Jan / Endur'O team,Coddy,Cathy,Earthood,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C128" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Deadlines are dates. Leave blank if no date is set yet." type="date" operator="greaterThan">
       <formula1>DATE(2024,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2952,7 +2992,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Seeded 2026-09-26 from 127 actions by tools/make_owner_workbook.py</t>
+          <t>Seeded 2026-09-28 from 129 actions by tools/make_owner_workbook.py</t>
         </is>
       </c>
     </row>

</xml_diff>